<commit_message>
docs(cwms): slate change — Zach dual-hats Forms Dev + Oracle DBA (Q&A 9), Efrain removed; pricing/xlsx/LOCs/org chart updated; rebuild
</commit_message>
<xml_diff>
--- a/docs/responses/2026-09-03-usace-cwms-authz/out/Vol-III-Price-FrasierDigital.xlsx
+++ b/docs/responses/2026-09-03-usace-cwms-authz/out/Vol-III-Price-FrasierDigital.xlsx
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="F6" s="5">
-        <f>'Hours by Task'!M4</f>
+        <f>'Hours by Task'!L4</f>
         <v/>
       </c>
     </row>
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="F7" s="5">
-        <f>'Hours by Task'!M5</f>
+        <f>'Hours by Task'!L5</f>
         <v/>
       </c>
     </row>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="F8" s="5">
-        <f>'Hours by Task'!M6</f>
+        <f>'Hours by Task'!L6</f>
         <v/>
       </c>
     </row>
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="F9" s="5">
-        <f>'Hours by Task'!M7</f>
+        <f>'Hours by Task'!L7</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="F10" s="5">
-        <f>'Hours by Task'!M8</f>
+        <f>'Hours by Task'!L8</f>
         <v/>
       </c>
     </row>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="F11" s="5">
-        <f>'Hours by Task'!M9</f>
+        <f>'Hours by Task'!L9</f>
         <v/>
       </c>
     </row>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="F12" s="5">
-        <f>'Hours by Task'!M10</f>
+        <f>'Hours by Task'!L10</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="F13" s="5">
-        <f>'Hours by Task'!M11</f>
+        <f>'Hours by Task'!L11</f>
         <v/>
       </c>
     </row>
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -877,12 +877,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>E. Rocha</t>
+          <t>S. Carpenter</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Senior Oracle DBA</t>
+          <t>System Engineer / Architect</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -897,12 +897,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>S. Carpenter</t>
+          <t>Z. Antosko</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>System Engineer / Architect</t>
+          <t>Senior Forms (React/TypeScript) Developer / Senior Oracle DBA (dual role)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -917,12 +917,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Z. Antosko</t>
+          <t>R. Chong</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Senior Forms (React/TypeScript) Developer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -937,27 +937,27 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>R. Chong</t>
+          <t>A. Frasier</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Associate Software Engineer</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>A. Frasier</t>
+          <t>S. Chesky</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -971,26 +971,6 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>S. Chesky</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Associate Software Engineer</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n">
         <v>90</v>
       </c>
     </row>
@@ -1005,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1019,8 +999,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1058,40 +1037,35 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>E. Rocha</t>
+          <t>S. Carpenter</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>S. Carpenter</t>
+          <t>Z. Antosko</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Z. Antosko</t>
+          <t>R. Chong</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>R. Chong</t>
+          <t>A. Frasier</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>A. Frasier</t>
+          <t>S. Chesky</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>S. Chesky</t>
+          <t>Total hours</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Total hours</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Task price</t>
         </is>
@@ -1122,29 +1096,26 @@
         <v>78</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>12</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="4">
-        <f>SUM(E4:K4)</f>
-        <v/>
-      </c>
-      <c r="M4" s="5">
-        <f>E4*'Labor Rates'!$D$5+F4*'Labor Rates'!$D$6+G4*'Labor Rates'!$D$7+H4*'Labor Rates'!$D$8+I4*'Labor Rates'!$D$9+J4*'Labor Rates'!$D$10+K4*'Labor Rates'!$D$11</f>
+      <c r="K4" s="4">
+        <f>SUM(E4:J4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="5">
+        <f>E4*'Labor Rates'!$D$5+F4*'Labor Rates'!$D$6+G4*'Labor Rates'!$D$7+H4*'Labor Rates'!$D$8+I4*'Labor Rates'!$D$9+J4*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1173,29 +1144,26 @@
         <v>50</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G5" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="4" t="n">
-        <v>220</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="4">
-        <f>SUM(E5:K5)</f>
-        <v/>
-      </c>
-      <c r="M5" s="5">
-        <f>E5*'Labor Rates'!$D$5+F5*'Labor Rates'!$D$6+G5*'Labor Rates'!$D$7+H5*'Labor Rates'!$D$8+I5*'Labor Rates'!$D$9+J5*'Labor Rates'!$D$10+K5*'Labor Rates'!$D$11</f>
+      <c r="K5" s="4">
+        <f>SUM(E5:J5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="5">
+        <f>E5*'Labor Rates'!$D$5+F5*'Labor Rates'!$D$6+G5*'Labor Rates'!$D$7+H5*'Labor Rates'!$D$8+I5*'Labor Rates'!$D$9+J5*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1224,29 +1192,26 @@
         <v>40</v>
       </c>
       <c r="F6" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="4" t="n">
-        <v>120</v>
-      </c>
       <c r="H6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="I6" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>40</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="4">
-        <f>SUM(E6:K6)</f>
-        <v/>
-      </c>
-      <c r="M6" s="5">
-        <f>E6*'Labor Rates'!$D$5+F6*'Labor Rates'!$D$6+G6*'Labor Rates'!$D$7+H6*'Labor Rates'!$D$8+I6*'Labor Rates'!$D$9+J6*'Labor Rates'!$D$10+K6*'Labor Rates'!$D$11</f>
+      <c r="K6" s="4">
+        <f>SUM(E6:J6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="5">
+        <f>E6*'Labor Rates'!$D$5+F6*'Labor Rates'!$D$6+G6*'Labor Rates'!$D$7+H6*'Labor Rates'!$D$8+I6*'Labor Rates'!$D$9+J6*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1275,29 +1240,26 @@
         <v>70</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="I7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>150</v>
-      </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="4" t="n">
         <v>400</v>
       </c>
-      <c r="L7" s="4">
-        <f>SUM(E7:K7)</f>
-        <v/>
-      </c>
-      <c r="M7" s="5">
-        <f>E7*'Labor Rates'!$D$5+F7*'Labor Rates'!$D$6+G7*'Labor Rates'!$D$7+H7*'Labor Rates'!$D$8+I7*'Labor Rates'!$D$9+J7*'Labor Rates'!$D$10+K7*'Labor Rates'!$D$11</f>
+      <c r="K7" s="4">
+        <f>SUM(E7:J7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="5">
+        <f>E7*'Labor Rates'!$D$5+F7*'Labor Rates'!$D$6+G7*'Labor Rates'!$D$7+H7*'Labor Rates'!$D$8+I7*'Labor Rates'!$D$9+J7*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1326,29 +1288,26 @@
         <v>78</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>12</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L8" s="4">
-        <f>SUM(E8:K8)</f>
-        <v/>
-      </c>
-      <c r="M8" s="5">
-        <f>E8*'Labor Rates'!$D$5+F8*'Labor Rates'!$D$6+G8*'Labor Rates'!$D$7+H8*'Labor Rates'!$D$8+I8*'Labor Rates'!$D$9+J8*'Labor Rates'!$D$10+K8*'Labor Rates'!$D$11</f>
+      <c r="K8" s="4">
+        <f>SUM(E8:J8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="5">
+        <f>E8*'Labor Rates'!$D$5+F8*'Labor Rates'!$D$6+G8*'Labor Rates'!$D$7+H8*'Labor Rates'!$D$8+I8*'Labor Rates'!$D$9+J8*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1377,29 +1336,26 @@
         <v>20</v>
       </c>
       <c r="F9" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="4" t="n">
-        <v>80</v>
-      </c>
       <c r="H9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="4">
-        <f>SUM(E9:K9)</f>
-        <v/>
-      </c>
-      <c r="M9" s="5">
-        <f>E9*'Labor Rates'!$D$5+F9*'Labor Rates'!$D$6+G9*'Labor Rates'!$D$7+H9*'Labor Rates'!$D$8+I9*'Labor Rates'!$D$9+J9*'Labor Rates'!$D$10+K9*'Labor Rates'!$D$11</f>
+      <c r="K9" s="4">
+        <f>SUM(E9:J9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="5">
+        <f>E9*'Labor Rates'!$D$5+F9*'Labor Rates'!$D$6+G9*'Labor Rates'!$D$7+H9*'Labor Rates'!$D$8+I9*'Labor Rates'!$D$9+J9*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1428,29 +1384,26 @@
         <v>20</v>
       </c>
       <c r="F10" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G10" s="4" t="n">
-        <v>60</v>
-      </c>
       <c r="H10" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="I10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="L10" s="4">
-        <f>SUM(E10:K10)</f>
-        <v/>
-      </c>
-      <c r="M10" s="5">
-        <f>E10*'Labor Rates'!$D$5+F10*'Labor Rates'!$D$6+G10*'Labor Rates'!$D$7+H10*'Labor Rates'!$D$8+I10*'Labor Rates'!$D$9+J10*'Labor Rates'!$D$10+K10*'Labor Rates'!$D$11</f>
+      <c r="K10" s="4">
+        <f>SUM(E10:J10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="5">
+        <f>E10*'Labor Rates'!$D$5+F10*'Labor Rates'!$D$6+G10*'Labor Rates'!$D$7+H10*'Labor Rates'!$D$8+I10*'Labor Rates'!$D$9+J10*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1479,29 +1432,26 @@
         <v>60</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G11" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="I11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="4" t="n">
-        <v>90</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>130</v>
-      </c>
       <c r="J11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="4" t="n">
         <v>350</v>
       </c>
-      <c r="L11" s="4">
-        <f>SUM(E11:K11)</f>
-        <v/>
-      </c>
-      <c r="M11" s="5">
-        <f>E11*'Labor Rates'!$D$5+F11*'Labor Rates'!$D$6+G11*'Labor Rates'!$D$7+H11*'Labor Rates'!$D$8+I11*'Labor Rates'!$D$9+J11*'Labor Rates'!$D$10+K11*'Labor Rates'!$D$11</f>
+      <c r="K11" s="4">
+        <f>SUM(E11:J11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="5">
+        <f>E11*'Labor Rates'!$D$5+F11*'Labor Rates'!$D$6+G11*'Labor Rates'!$D$7+H11*'Labor Rates'!$D$8+I11*'Labor Rates'!$D$9+J11*'Labor Rates'!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1542,12 +1492,8 @@
         <f>SUM(K4:K11)</f>
         <v/>
       </c>
-      <c r="L12" s="3">
+      <c r="L12" s="6">
         <f>SUM(L4:L11)</f>
-        <v/>
-      </c>
-      <c r="M12" s="6">
-        <f>SUM(M4:M11)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(cwms): slate v3 — Ryan Daley=Sr Forms Dev, Randy=Java+Oracle DBA dual (Zach unreachable); rebuild, new LOC PDFs
</commit_message>
<xml_diff>
--- a/docs/responses/2026-09-03-usace-cwms-authz/out/Vol-III-Price-FrasierDigital.xlsx
+++ b/docs/responses/2026-09-03-usace-cwms-authz/out/Vol-III-Price-FrasierDigital.xlsx
@@ -897,12 +897,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Z. Antosko</t>
+          <t>R. Daley</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Senior Forms (React/TypeScript) Developer / Senior Oracle DBA (dual role)</t>
+          <t>Senior Forms (React/TypeScript) Developer</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Senior Java Developer / Senior Oracle DBA (dual role)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Z. Antosko</t>
+          <t>R. Daley</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1099,10 +1099,10 @@
         <v>12</v>
       </c>
       <c r="G4" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" s="4" t="n">
         <v>20</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>0</v>
@@ -1147,10 +1147,10 @@
         <v>0</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="I5" s="4" t="n">
         <v>100</v>
@@ -1243,10 +1243,10 @@
         <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>0</v>
@@ -1291,10 +1291,10 @@
         <v>12</v>
       </c>
       <c r="G8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>20</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>0</v>
@@ -1387,10 +1387,10 @@
         <v>60</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>0</v>
@@ -1435,10 +1435,10 @@
         <v>0</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="I11" s="4" t="n">
         <v>0</v>

</xml_diff>